<commit_message>
feat: add quote_date to template, model, parser and import display
</commit_message>
<xml_diff>
--- a/frontend/template/import_template.xlsx
+++ b/frontend/template/import_template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="报价导入模板" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'报价导入模板'!$A$1:$L$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'报价导入模板'!$A$1:$M$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -78,12 +80,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -451,21 +456,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -491,40 +497,45 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>报价日期</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>产品/服务名称</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>设备型号</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>单位</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>单价</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>币种</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>产品类别</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>品牌/备注</t>
         </is>
@@ -551,38 +562,43 @@
           <t>info@promise.com.mo</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>紧急呼叫系统网关 Telligence Station Gateway</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>NGGTWY2-HNGGWPWR-AK</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="J2" s="2" t="n">
         <v>48220</v>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>MOP</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>呼叫/报警系统</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Ascom</t>
         </is>
@@ -609,38 +625,43 @@
           <t>zhang@hikvision.com</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>泊车识别摄像机 DS-TCP440-B</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>DS-TCP440-B</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="J3" s="2" t="n">
         <v>1810</v>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>MOP</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>安防摄像头</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Hikvision / 大华可选</t>
         </is>
@@ -651,46 +672,51 @@
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>智能停车场管理终端机 DS-TPM400-FP</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>DS-TPM400-FP</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="J4" s="2" t="n">
         <v>10760</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>MOP</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>停车系统</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L13"/>
+  <autoFilter ref="A1:M13"/>
   <dataValidations count="2">
-    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效币种" error="请选择 CNY / HKD / MOP" type="list">
+    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效币种" error="请选择 CNY / HKD / MOP" type="list">
       <formula1>"CNY,HKD,MOP"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效类别" error="请从下拉列表选择产品类别" type="list">
+    <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="无效类别" error="请从下拉列表选择产品类别" type="list">
       <formula1>"安防摄像头,门禁系统,网络设备,呼叫/报警系统,停车系统,软件/服务器,显示设备,机柜/配件,线缆/管材,电源设备,广播/音响,对讲系统,其他设备"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>